<commit_message>
MAJ pipeline 2026-09-23 14:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-09-23.xlsx
+++ b/jira_export_2026-09-23.xlsx
@@ -1405,9 +1405,9 @@
         </is>
       </c>
       <c r="N9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="12" t="n">
+        <v>600</v>
+      </c>
+      <c r="O9" s="16" t="n">
         <v>0</v>
       </c>
       <c r="P9" s="12" t="n">
@@ -13007,7 +13007,7 @@
       <c r="L176" s="17" t="inlineStr"/>
       <c r="M176" s="17" t="inlineStr"/>
       <c r="N176" s="18" t="n">
-        <v>47982.22500000001</v>
+        <v>48582.22500000001</v>
       </c>
       <c r="O176" s="18" t="n">
         <v>42930.25800000001</v>

</xml_diff>